<commit_message>
docs: add M2b peer z-score reverse engineering
</commit_message>
<xml_diff>
--- a/docs/M2_PV_Performance_Workbook.xlsx
+++ b/docs/M2_PV_Performance_Workbook.xlsx
@@ -75,7 +75,7 @@
     <definedName name="rstr_fleet_mean">M2b_PeerZScore!$B$15</definedName>
     <definedName name="rstr_fleet_median">M2b_PeerZScore!$B$16</definedName>
     <definedName name="rstr_fleet_std">M2b_PeerZScore!$B$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Findings_Summary'!$A$4:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Findings_Summary'!$A$4:$H$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5636,22 +5636,10 @@
         <f>IFERROR((B10-rstr_fleet_median)/rstr_fleet_std,"")</f>
         <v/>
       </c>
-      <c r="D26" s="15">
-        <f>IF(cfg_stat_method="median",C26,IF(cfg_stat_method="mean",B26,IF(ABS(B26)&gt;=ABS(C26),B26,C26)))</f>
-        <v/>
-      </c>
-      <c r="E26" s="5">
-        <f>IF(ABS(D26)&gt;cfg_z_threshold,1,0)</f>
-        <v/>
-      </c>
-      <c r="F26" s="5">
-        <f>IFERROR(IF(E10&gt;cfg_voc_ratio_threshold,1,0),0)</f>
-        <v/>
-      </c>
-      <c r="G26" s="5">
-        <f>IF(AND(E26=1,F26=1),1,0)</f>
-        <v/>
-      </c>
+      <c r="D26" s="15" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5">
         <f>IF(G26=1,"high_R","")</f>
         <v/>
@@ -6452,7 +6440,7 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Note: window 15 butuh ≥15 samples. Dummy 24 timestep cukup untuk demo.</t>
+          <t>Note: rolling_MAD pakai AVEDEV (mean-abs-dev) = proxy MAD universal-compatible (MEDIAN(IF()) array gagal tanpa CSE di LibreOffice). True Hampel = median-abs-dev x 1.4826; AVEDEV strict ~1.2533. Demo mekanisme, bukan filter produksi (preprocessing.py pakai pvanalytics).</t>
         </is>
       </c>
     </row>
@@ -6516,7 +6504,7 @@
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>MEDIAN(IF(B6:B6&gt;0,ABS(B6:B6-C6)))</f>
+        <f>AVEDEV(B6:B6)</f>
         <v/>
       </c>
       <c r="F6" s="15">
@@ -6550,7 +6538,7 @@
         <v/>
       </c>
       <c r="E7" s="15">
-        <f>MEDIAN(IF(B6:B7&gt;0,ABS(B6:B7-C7)))</f>
+        <f>AVEDEV(B6:B7)</f>
         <v/>
       </c>
       <c r="F7" s="15">
@@ -6584,7 +6572,7 @@
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>MEDIAN(IF(B6:B8&gt;0,ABS(B6:B8-C8)))</f>
+        <f>AVEDEV(B6:B8)</f>
         <v/>
       </c>
       <c r="F8" s="15">
@@ -6618,7 +6606,7 @@
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>MEDIAN(IF(B6:B9&gt;0,ABS(B6:B9-C9)))</f>
+        <f>AVEDEV(B6:B9)</f>
         <v/>
       </c>
       <c r="F9" s="15">
@@ -6652,7 +6640,7 @@
         <v/>
       </c>
       <c r="E10" s="15">
-        <f>MEDIAN(IF(B6:B10&gt;0,ABS(B6:B10-C10)))</f>
+        <f>AVEDEV(B6:B10)</f>
         <v/>
       </c>
       <c r="F10" s="15">
@@ -6686,7 +6674,7 @@
         <v/>
       </c>
       <c r="E11" s="15">
-        <f>MEDIAN(IF(B6:B11&gt;0,ABS(B6:B11-C11)))</f>
+        <f>AVEDEV(B6:B11)</f>
         <v/>
       </c>
       <c r="F11" s="15">
@@ -6720,7 +6708,7 @@
         <v/>
       </c>
       <c r="E12" s="15">
-        <f>MEDIAN(IF(B6:B12&gt;0,ABS(B6:B12-C12)))</f>
+        <f>AVEDEV(B6:B12)</f>
         <v/>
       </c>
       <c r="F12" s="15">
@@ -6754,7 +6742,7 @@
         <v/>
       </c>
       <c r="E13" s="15">
-        <f>MEDIAN(IF(B6:B13&gt;0,ABS(B6:B13-C13)))</f>
+        <f>AVEDEV(B6:B13)</f>
         <v/>
       </c>
       <c r="F13" s="15">
@@ -6788,7 +6776,7 @@
         <v/>
       </c>
       <c r="E14" s="15">
-        <f>MEDIAN(IF(B6:B14&gt;0,ABS(B6:B14-C14)))</f>
+        <f>AVEDEV(B6:B14)</f>
         <v/>
       </c>
       <c r="F14" s="15">
@@ -6822,7 +6810,7 @@
         <v/>
       </c>
       <c r="E15" s="15">
-        <f>MEDIAN(IF(B6:B15&gt;0,ABS(B6:B15-C15)))</f>
+        <f>AVEDEV(B6:B15)</f>
         <v/>
       </c>
       <c r="F15" s="15">
@@ -6856,7 +6844,7 @@
         <v/>
       </c>
       <c r="E16" s="15">
-        <f>MEDIAN(IF(B6:B16&gt;0,ABS(B6:B16-C16)))</f>
+        <f>AVEDEV(B6:B16)</f>
         <v/>
       </c>
       <c r="F16" s="15">
@@ -6890,7 +6878,7 @@
         <v/>
       </c>
       <c r="E17" s="15">
-        <f>MEDIAN(IF(B6:B17&gt;0,ABS(B6:B17-C17)))</f>
+        <f>AVEDEV(B6:B17)</f>
         <v/>
       </c>
       <c r="F17" s="15">
@@ -6924,7 +6912,7 @@
         <v/>
       </c>
       <c r="E18" s="15">
-        <f>MEDIAN(IF(B6:B18&gt;0,ABS(B6:B18-C18)))</f>
+        <f>AVEDEV(B6:B18)</f>
         <v/>
       </c>
       <c r="F18" s="15">
@@ -6958,7 +6946,7 @@
         <v/>
       </c>
       <c r="E19" s="15">
-        <f>MEDIAN(IF(B6:B19&gt;0,ABS(B6:B19-C19)))</f>
+        <f>AVEDEV(B6:B19)</f>
         <v/>
       </c>
       <c r="F19" s="15">
@@ -6992,7 +6980,7 @@
         <v/>
       </c>
       <c r="E20" s="15">
-        <f>MEDIAN(IF(B6:B20&gt;0,ABS(B6:B20-C20)))</f>
+        <f>AVEDEV(B6:B20)</f>
         <v/>
       </c>
       <c r="F20" s="15">
@@ -7026,7 +7014,7 @@
         <v/>
       </c>
       <c r="E21" s="15">
-        <f>MEDIAN(IF(B7:B21&gt;0,ABS(B7:B21-C21)))</f>
+        <f>AVEDEV(B7:B21)</f>
         <v/>
       </c>
       <c r="F21" s="15">
@@ -7060,7 +7048,7 @@
         <v/>
       </c>
       <c r="E22" s="15">
-        <f>MEDIAN(IF(B8:B22&gt;0,ABS(B8:B22-C22)))</f>
+        <f>AVEDEV(B8:B22)</f>
         <v/>
       </c>
       <c r="F22" s="15">
@@ -7094,7 +7082,7 @@
         <v/>
       </c>
       <c r="E23" s="15">
-        <f>MEDIAN(IF(B9:B23&gt;0,ABS(B9:B23-C23)))</f>
+        <f>AVEDEV(B9:B23)</f>
         <v/>
       </c>
       <c r="F23" s="15">
@@ -7128,7 +7116,7 @@
         <v/>
       </c>
       <c r="E24" s="15">
-        <f>MEDIAN(IF(B10:B24&gt;0,ABS(B10:B24-C24)))</f>
+        <f>AVEDEV(B10:B24)</f>
         <v/>
       </c>
       <c r="F24" s="15">
@@ -7162,7 +7150,7 @@
         <v/>
       </c>
       <c r="E25" s="15">
-        <f>MEDIAN(IF(B11:B25&gt;0,ABS(B11:B25-C25)))</f>
+        <f>AVEDEV(B11:B25)</f>
         <v/>
       </c>
       <c r="F25" s="15">
@@ -7196,7 +7184,7 @@
         <v/>
       </c>
       <c r="E26" s="15">
-        <f>MEDIAN(IF(B12:B26&gt;0,ABS(B12:B26-C26)))</f>
+        <f>AVEDEV(B12:B26)</f>
         <v/>
       </c>
       <c r="F26" s="15">
@@ -7230,7 +7218,7 @@
         <v/>
       </c>
       <c r="E27" s="15">
-        <f>MEDIAN(IF(B13:B27&gt;0,ABS(B13:B27-C27)))</f>
+        <f>AVEDEV(B13:B27)</f>
         <v/>
       </c>
       <c r="F27" s="15">
@@ -7264,7 +7252,7 @@
         <v/>
       </c>
       <c r="E28" s="15">
-        <f>MEDIAN(IF(B14:B28&gt;0,ABS(B14:B28-C28)))</f>
+        <f>AVEDEV(B14:B28)</f>
         <v/>
       </c>
       <c r="F28" s="15">
@@ -7298,7 +7286,7 @@
         <v/>
       </c>
       <c r="E29" s="15">
-        <f>MEDIAN(IF(B15:B29&gt;0,ABS(B15:B29-C29)))</f>
+        <f>AVEDEV(B15:B29)</f>
         <v/>
       </c>
       <c r="F29" s="15">
@@ -13728,7 +13716,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H22"/>
+  <autoFilter ref="A4:H21"/>
   <conditionalFormatting sqref="E5:E16">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"CRITICAL"</formula>
@@ -13752,7 +13740,7 @@
       <formula>"NO_DAYLIGHT"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E22">
+  <conditionalFormatting sqref="E5:E21">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="0">
       <formula>"CRITICAL"</formula>
     </cfRule>

</xml_diff>